<commit_message>
feat: identify AI questions with five-digit tags
</commit_message>
<xml_diff>
--- a/考试配置表.xlsx
+++ b/考试配置表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="考试设置" sheetId="1" r:id="Rcf24a4df67d24912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选题明细" sheetId="2" r:id="R36f85cc6cfe84f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="考试设置" sheetId="1" r:id="R019df10ca4004090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选题明细" sheetId="2" r:id="Rb95407b6caa14829"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,16 +116,7 @@
     <x:t xml:space="preserve">章内题目编号</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">题干关键词（核对用）</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">分值（可选）</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">复指数信号</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">周期信号</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">填写规则</x:t>
@@ -615,11 +606,11 @@
       <x:c r="C1" s="2" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D1" s="2" t="s">
+      <x:c r="D1" s="2" t="str">
+        <x:v>五位唯一标识（核对用）</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="s">
-        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34.04999923706055" customHeight="1">
@@ -637,8 +628,8 @@
       <x:c r="C3" s="3">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="s">
-        <x:v>37</x:v>
+      <x:c r="D3" s="3" t="str">
+        <x:v>[10001]</x:v>
       </x:c>
       <x:c r="E3" s="3">
         <x:v>5</x:v>
@@ -652,8 +643,8 @@
       <x:c r="C4" s="1">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" s="1" t="s">
-        <x:v>38</x:v>
+      <x:c r="D4" s="1" t="str">
+        <x:v>[10002]</x:v>
       </x:c>
       <x:c r="E4" s="1">
         <x:v>5</x:v>
@@ -668,10 +659,10 @@
     </x:row>
     <x:row r="6" ht="34.04999923706055" customHeight="1">
       <x:c r="A6" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>40</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C6" s="6"/>
       <x:c r="D6" s="6"/>
@@ -679,10 +670,10 @@
     </x:row>
     <x:row r="7" ht="34.04999923706055" customHeight="1">
       <x:c r="A7" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>42</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -690,10 +681,10 @@
     </x:row>
     <x:row r="8" ht="34.04999923706055" customHeight="1">
       <x:c r="A8" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B8" s="6" t="s">
-        <x:v>44</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>

</xml_diff>

<commit_message>
feat: make chapter question number optional
</commit_message>
<xml_diff>
--- a/考试配置表.xlsx
+++ b/考试配置表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="考试设置" sheetId="1" r:id="R019df10ca4004090"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选题明细" sheetId="2" r:id="Rb95407b6caa14829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="考试设置" sheetId="1" r:id="Re174e7c4cc3a4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选题明细" sheetId="2" r:id="R86c475a5dfa440b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -111,9 +111,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">章节名称（核对用）</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">章内题目编号</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">分值（可选）</x:t>
@@ -603,14 +600,14 @@
       <x:c r="B1" s="2" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>34</x:v>
+      <x:c r="C1" s="2" t="str">
+        <x:v>章内题目编号（可留空）</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
         <x:v>五位唯一标识（核对用）</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34.04999923706055" customHeight="1">
@@ -659,10 +656,10 @@
     </x:row>
     <x:row r="6" ht="34.04999923706055" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="s">
         <x:v>36</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>37</x:v>
       </x:c>
       <x:c r="C6" s="6"/>
       <x:c r="D6" s="6"/>
@@ -670,10 +667,10 @@
     </x:row>
     <x:row r="7" ht="34.04999923706055" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
         <x:v>38</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>39</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -681,10 +678,10 @@
     </x:row>
     <x:row r="8" ht="34.04999923706055" customHeight="1">
       <x:c r="A8" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>

</xml_diff>